<commit_message>
Log v3 equation smoke test
</commit_message>
<xml_diff>
--- a/CANON_TEST_LEDGER/THEOPHYSICS_TEST_LEDGER.xlsx
+++ b/CANON_TEST_LEDGER/THEOPHYSICS_TEST_LEDGER.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K61"/>
+  <dimension ref="A1:K62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2933,6 +2933,63 @@
       <c r="I61" s="2" t="inlineStr"/>
       <c r="J61" s="2" t="inlineStr"/>
       <c r="K61" s="2" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>T061</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>TEST-0000-v3-equation-smoke</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>PYTHON</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>V3_SMOKE</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Smallest executable gate for the v3 Master Equation adapter: 9-factor domain, product chi, analytic gradient, zero-veto precision, dX/dt wiring, and rejection of old 10-factor shape.</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>Passed local Python compile and execution on 2026-07-27. This verifies the executable equation adapter only; it is not a Lean proof, empirical validation, or full Lagrangian benchmark.</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/DavidLoweOKC/theophysics-prediction-lab/tree/main/v3-tests/TEST-0000-v3-equation-smoke</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>Commit 257856b. Output artifact: outputs/smoke_output_20260727.txt. Next step: comparative Lagrangian bench with controls + historical equation + v3 canonical equation.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6293,9 +6350,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -6310,9 +6365,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -6362,9 +6415,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr"/>
-    </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Log comparative Lagrangian v3 bench
</commit_message>
<xml_diff>
--- a/CANON_TEST_LEDGER/THEOPHYSICS_TEST_LEDGER.xlsx
+++ b/CANON_TEST_LEDGER/THEOPHYSICS_TEST_LEDGER.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K62"/>
+  <dimension ref="A1:K63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2988,6 +2988,63 @@
       <c r="K62" s="2" t="inlineStr">
         <is>
           <t>Commit 257856b. Output artifact: outputs/smoke_output_20260727.txt. Next step: comparative Lagrangian bench with controls + historical equation + v3 canonical equation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>T062</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>TEST-0001-comparative-lagrangian-bench</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>PYTHON</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>V3_LAGRANGIAN</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>Focused side-by-side Lagrangian migration bench: standard controls + HISTORICAL_EQUATION_SLOT + V3_CANONICAL_EQUATION_SLOT under shared finite-value, mass-matrix, short-integration, and equation-slot checks.</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>Passed local Python compile and execution on 2026-07-27. Controls passed 10/10 combined; Historical L1 passed 8/8 as historical comparison; V3 canonical model passed 11/11. This is a compatibility/migration bench, not final LLC proof or Law 5/Law 9 reproduction.</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/DavidLoweOKC/theophysics-prediction-lab/tree/main/v3-tests/TEST-0001-comparative-lagrangian-bench</t>
+        </is>
+      </c>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>Commit 613e557. Output artifacts: outputs/results.json, outputs/summary.csv, outputs/bench_output_20260727.txt. Next step: larger historical bench or Family Lagrangian applied-domain packet.</t>
         </is>
       </c>
     </row>
@@ -6350,7 +6407,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -6365,7 +6421,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -6415,7 +6470,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>

</xml_diff>